<commit_message>
Add SERP theme context to every cluster
Per-cluster analyst-written context from live top-10 data: who ranks,
winning page format, and dominant intent. Propagated to clusters.xlsx,
cluster-head-terms.xlsx, clusters.csv/json, and the explorer.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01RMLqY5quomFqhwKV9guW8U
</commit_message>
<xml_diff>
--- a/igaming/cluster-head-terms.xlsx
+++ b/igaming/cluster-head-terms.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Cluster Head Terms" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Cluster Head Terms'!$A$1:$D$103</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Cluster Head Terms'!$A$1:$G$103</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -63,12 +63,17 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
+      <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -434,13 +439,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D103"/>
+  <dimension ref="A1:G103"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="46" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="80" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="26" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -464,6 +472,21 @@
           <t>Cluster total volume</t>
         </is>
       </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>SERP theme</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Winning format</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>SERP intent</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -480,6 +503,21 @@
       <c r="D2" s="2" t="n">
         <v>7350</v>
       </c>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>Fragmented SERP: Indeed job listings (DR92), Sportradar's marketing-services product page, agency strategy blog posts (DataArt, low-DR Team Catalyst DR5), an academic NIH paper and an agency listicle, with a Medium UGC post in the top 10. No single format owns the query.</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>mixed/fragmented</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>mixed</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -496,6 +534,21 @@
       <c r="D3" s="2" t="n">
         <v>6010</v>
       </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>Affiliate program directories and listicles dominate (BusinessofApps, AffPaying, AskGamblers, StatsDrone) alongside program operators' own homepages (Alpha Affiliates, LivePartners) and an ad-network blog listicle (RichAds). Reddit at #3 and YouTube in the top 10 show Google rewarding UGC here.</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>program directory / listicle</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>join affiliate program</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -512,6 +565,21 @@
       <c r="D4" s="2" t="n">
         <v>4840</v>
       </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>Affiliate-SaaS vendors win with blog guides and comparison posts (Tracknow, iRev, Voluum, Affise) plus product homepages (Affilka); a DR6 exact-match domain (igamingaffiliates.io) ranks #2, signalling a beatable SERP.</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>vendor blog guide</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>choose vendor/tool</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -528,6 +596,21 @@
       <c r="D5" s="2" t="n">
         <v>3210</v>
       </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>How-to guides and program listicles from ad-network/tracker blogs (RichAds, Voluum) and affiliate directories (BusinessofApps, StatsDrone, BettingUSA) fill the page; Reddit holds #1 and YouTube also ranks, a clear UGC weakness.</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>how-to guide / listicle</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>learn / how-to</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -544,6 +627,21 @@
       <c r="D6" s="2" t="n">
         <v>1640</v>
       </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>High-DR news outlets (Guardian, ESPN), industry-association trend reports (American Gaming Association), and academic/ethics pieces (NIH, Brooklyn Law) own the SERP; nothing commercial ranks and Reddit sits mid-page.</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>news / research articles</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>industry reference</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -560,6 +658,21 @@
       <c r="D7" s="2" t="n">
         <v>1520</v>
       </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>Split between iGaming agency landing pages (Luvkaizen DR28, igaming.agency DR0.7, ICS Digital) and 'top agencies' listicles (Absolute Digital, HilltopAds, DR10 Redclawey); many low-DR domains plus a LinkedIn company page in the top 10 make this a soft SERP.</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>agency landing page / listicle</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>choose vendor/tool</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -576,6 +689,21 @@
       <c r="D8" s="2" t="n">
         <v>1510</v>
       </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>Consumer-facing SERP: Reddit complaints at #1, GambleAware and UK Gambling Commission pages on limiting/opting out of gambling ads, Wikipedia, and news coverage. Searchers here are mostly annoyed consumers, not advertisers.</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>mixed/fragmented</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>mixed</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -592,6 +720,21 @@
       <c r="D9" s="2" t="n">
         <v>1390</v>
       </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>iGaming SEO agency landing pages dominate, mostly low-DR (tbd.media DR27, Qwerty Labs DR15, Naturallinks DR38) alongside GeekyTech (DR75); Trustpilot and a LinkedIn company page also rank, confirming a weak, winnable SERP.</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>agency landing page</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>choose vendor/tool</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -608,6 +751,21 @@
       <c r="D10" s="2" t="n">
         <v>1210</v>
       </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>Policy and reference pages rule: Google Ads and Meta ad-policy documentation, UK Parliament research briefing, Wikipedia, AGA ad-spend PDF and news; Reddit appears mid-page. All-high-DR institutional SERP with no commercial players.</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>policy documentation</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>policy / compliance reference</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -624,6 +782,21 @@
       <c r="D11" s="2" t="n">
         <v>1190</v>
       </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>Land-based-leaning mix of Indeed jobs (#1), how-to guides from martech blogs (iPost, MoEngage, Cvent) and casino agency pages (Good Giant, LT Agency, DR7 Casino Marketing Bootcamp); a LinkedIn page also ranks.</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>how-to guide</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>learn / how-to</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -640,6 +813,21 @@
       <c r="D12" s="2" t="n">
         <v>980</v>
       </c>
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t>Agency directories are the power players (Semrush Agencies DR92, Clutch DR91, Influencer Marketing Hub) interleaved with individual agency landing pages (Bird, LT Agency, Straight North, low-DR Velocity/Good Giant) and a LinkedIn UGC result.</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>agency directory / listicle</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>choose vendor/tool</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -656,6 +844,21 @@
       <c r="D13" s="2" t="n">
         <v>820</v>
       </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>Highly fragmented: an agency landing page, tactic articles on niche industry sites (WA Technology, DR21 Grou Global), a HilltopAds listicle, job pages (ZipRecruiter, DR1.7 igamingcareers) and LinkedIn Pulse UGC. Several sub-DR30 domains rank — weak SERP with unsettled intent.</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>mixed/fragmented</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>mixed</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -672,6 +875,21 @@
       <c r="D14" s="2" t="n">
         <v>750</v>
       </c>
+      <c r="E14" s="3" t="inlineStr">
+        <is>
+          <t>Step-by-step how-to guides from iGaming platform providers (SoftGamings, Sirplay, Genome, iGamingBusiness/TrueLabel, RichAds) and a law-services explainer; Reddit holds #1, exposing a UGC gap.</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>how-to guide</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>learn / how-to</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -688,6 +906,21 @@
       <c r="D15" s="2" t="n">
         <v>710</v>
       </c>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>Google's own policy doc at #2, followed by blockchain-ads.com's post at #3, industry news coverage (MediaPost, SBC Americas, Bettors Insider) and a RichAds blog post; YouTube and Reddit round out the top 10. News-plus-policy SERP where BCA already ranks.</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>news + policy doc</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>policy / compliance reference</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -704,6 +937,21 @@
       <c r="D16" s="2" t="n">
         <v>670</v>
       </c>
+      <c r="E16" s="3" t="inlineStr">
+        <is>
+          <t>Ad networks win with dedicated traffic landing pages and blog guides (RichAds /igaming-traffic, TrafficNomads DR27, Voluum, AffPapa guide, low-DR Z2A Digital); Reddit and YouTube both sit in the top 10 — a buyable SERP with UGC softness.</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>ad-network landing page / blog</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>buy traffic / choose platform</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -720,6 +968,21 @@
       <c r="D17" s="2" t="n">
         <v>480</v>
       </c>
+      <c r="E17" s="3" t="inlineStr">
+        <is>
+          <t>Creative-inspiration SERP: example galleries (Pinterest, Behance, Ads of the World, iSpot.tv) and campaign listicles (Everything-PR, RichAds creatives post) dominate, with heavy UGC (Pinterest, YouTube playlist) in the top 10.</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>creative example gallery / listicle</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>learn / how-to</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -736,6 +999,21 @@
       <c r="D18" s="2" t="n">
         <v>410</v>
       </c>
+      <c r="E18" s="3" t="inlineStr">
+        <is>
+          <t>CRM SaaS vendor product pages (Optimove, Solitics, Groovetech) and vendor listicles (DR25 OptiKPI) rank alongside Reddit and Medium UGC and very low-DR sites (DR4.4 Quettaspins) — a weak vendor-selection SERP.</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>product landing page / listicle</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>choose vendor/tool</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -752,6 +1030,21 @@
       <c r="D19" s="2" t="n">
         <v>400</v>
       </c>
+      <c r="E19" s="3" t="inlineStr">
+        <is>
+          <t>Platform policy pages top the SERP (Facebook Business Help #1, Meta ad standards, Google Ads policy), followed by promotion-tips listicles from vendors (Selzy, PartnerMatrix, RichAds ad-network listicle, BusinessofApps, Altenar). Compliance-first, then how-to.</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>policy pages + how-to listicle</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t>learn / how-to</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -768,6 +1061,21 @@
       <c r="D20" s="2" t="n">
         <v>400</v>
       </c>
+      <c r="E20" s="3" t="inlineStr">
+        <is>
+          <t>Affiliate-software vendors own the SERP with product pages (EveryMatrix PartnerMatrix #1, Affilka, Income Access) and vendor blog explainers (Track360 glossary, iRev, Smartico, Affise); solid mid-to-high DR throughout.</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>product landing page</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>choose vendor/tool</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -784,6 +1092,21 @@
       <c r="D21" s="2" t="n">
         <v>390</v>
       </c>
+      <c r="E21" s="3" t="inlineStr">
+        <is>
+          <t>UGC-riddled and fragmented: Pinterest boards at #1 and #4, a YouTube playlist, Wikipedia, plus a RichAds guide, an agency page (LT Agency) and a First Amendment law article. No commercial format has consolidated this SERP.</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>mixed/fragmented</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="inlineStr">
+        <is>
+          <t>mixed</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -800,6 +1123,21 @@
       <c r="D22" s="2" t="n">
         <v>370</v>
       </c>
+      <c r="E22" s="3" t="inlineStr">
+        <is>
+          <t>Idea/tips listicles on martech and vendor blogs win outright (Geotargetly, iPost, Odds On Promotions DR29, Selzy, Tegna, DR22 J Carcamo, MoEngage) — a classic listicle SERP with mostly mid-DR domains.</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>blog listicle</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>learn / how-to</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -816,6 +1154,21 @@
       <c r="D23" s="2" t="n">
         <v>350</v>
       </c>
+      <c r="E23" s="3" t="inlineStr">
+        <is>
+          <t>Definitional content wins: Wikipedia, glossary pages (Endava, Track-style), 'what is iGaming' guides (RichAds, Aeropay, Sportsbetting Dime, DR29 Global Advisory Experts), with Reddit and LinkedIn UGC also ranking.</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>definition guide / glossary</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="inlineStr">
+        <is>
+          <t>learn / how-to</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -832,6 +1185,21 @@
       <c r="D24" s="2" t="n">
         <v>310</v>
       </c>
+      <c r="E24" s="3" t="inlineStr">
+        <is>
+          <t>Ad networks and ad-tech blogs dominate: ReachEffect's iGaming LP at #1, Voluum and RichAds posts, BusinessofApps creative best practices, and blockchain-ads.com's iGaming ad examples post at #10; low-DR vizibl.ai (DR8) also ranks.</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>ad-network landing page / blog</t>
+        </is>
+      </c>
+      <c r="G24" s="2" t="inlineStr">
+        <is>
+          <t>buy traffic / choose platform</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -848,6 +1216,21 @@
       <c r="D25" s="2" t="n">
         <v>300</v>
       </c>
+      <c r="E25" s="3" t="inlineStr">
+        <is>
+          <t>Explainer guides from iGaming platform vendors (RichAds beginners guide, SoftSwiss, BetConstruct) mixed with the BusinessofApps directory and affiliate-program pages (PartnerMatrix, Affnook, Alpha Affiliates); Reddit sits mid-page.</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>how-to guide</t>
+        </is>
+      </c>
+      <c r="G25" s="2" t="inlineStr">
+        <is>
+          <t>learn / how-to</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -864,6 +1247,21 @@
       <c r="D26" s="2" t="n">
         <v>280</v>
       </c>
+      <c r="E26" s="3" t="inlineStr">
+        <is>
+          <t>Research-institution SERP: academic papers (NIH, ScienceDirect, ResearchGate-tier), UK Gambling Commission advertising rules, and industry PDFs (Responsible Gambling Council, AGA ad-spend). All high-DR; only Selzy, Elit-web and RichAds represent commercial content.</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>research / regulatory reports</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t>industry reference</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -880,6 +1278,21 @@
       <c r="D27" s="2" t="n">
         <v>220</v>
       </c>
+      <c r="E27" s="3" t="inlineStr">
+        <is>
+          <t>Academic and industry-research results lead (NIH #1, ResearchGate, AGA trend report) with strategy blog posts (DataArt, Elit-web) and Sportradar's product page mixed in — a reference-heavy SERP where commercial pages struggle above mid-page.</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>research + strategy blog</t>
+        </is>
+      </c>
+      <c r="G27" s="2" t="inlineStr">
+        <is>
+          <t>industry reference</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -896,6 +1309,21 @@
       <c r="D28" s="2" t="n">
         <v>210</v>
       </c>
+      <c r="E28" s="3" t="inlineStr">
+        <is>
+          <t>Program operators' signup pages win (LivePartners, Paddy Power Partnerships, Neto Partners) alongside directories (BusinessofApps) and guides (Track360, RichAds, SoftSwiss); a LinkedIn company page at #1 shows SERP weakness.</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>program signup pages</t>
+        </is>
+      </c>
+      <c r="G28" s="2" t="inlineStr">
+        <is>
+          <t>join affiliate program</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -912,6 +1340,21 @@
       <c r="D29" s="2" t="n">
         <v>200</v>
       </c>
+      <c r="E29" s="3" t="inlineStr">
+        <is>
+          <t>'Best iGaming ad networks' listicles on ad-network blogs win (Kadam, RichAds, DR12 AllinAffiliates, blockchain-ads.com's top-gambling-ad-networks at #10) plus network landing pages (ReachEffect #1, TrafficNomads); several sub-DR15 domains rank, including DR0 taroviser.</t>
+        </is>
+      </c>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>blog listicle</t>
+        </is>
+      </c>
+      <c r="G29" s="2" t="inlineStr">
+        <is>
+          <t>buy traffic / choose platform</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -928,6 +1371,21 @@
       <c r="D30" s="2" t="n">
         <v>200</v>
       </c>
+      <c r="E30" s="3" t="inlineStr">
+        <is>
+          <t>Comparison listicles on affiliate-SaaS vendor blogs dominate (iRev, Voluum, Trackdesk, Tracknow, Track360, DR30 aff.tech) with product pages (Everflow, EveryMatrix PartnerMatrix) filling out; Reddit ranks #4.</t>
+        </is>
+      </c>
+      <c r="F30" s="2" t="inlineStr">
+        <is>
+          <t>comparison listicle</t>
+        </is>
+      </c>
+      <c r="G30" s="2" t="inlineStr">
+        <is>
+          <t>choose vendor/tool</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -944,6 +1402,21 @@
       <c r="D31" s="2" t="n">
         <v>200</v>
       </c>
+      <c r="E31" s="3" t="inlineStr">
+        <is>
+          <t>Pure news SERP owned by top-tier outlets (BBC #1, Reuters, Washington Post, The Conversation) plus AGA and an NIH paper — uniformly very high DR, essentially unassailable without a news angle.</t>
+        </is>
+      </c>
+      <c r="F31" s="2" t="inlineStr">
+        <is>
+          <t>news articles</t>
+        </is>
+      </c>
+      <c r="G31" s="2" t="inlineStr">
+        <is>
+          <t>industry reference</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -960,6 +1433,21 @@
       <c r="D32" s="2" t="n">
         <v>190</v>
       </c>
+      <c r="E32" s="3" t="inlineStr">
+        <is>
+          <t>Ad networks win with vertical landing pages and how-to blogs (TrafficNomads DR27 at #1, Clickadu gambling-traffic LP, RichAds, Voluum, betting.partners); Reddit and a Semrush trending page also rank. Low-DR #1 signals an open SERP.</t>
+        </is>
+      </c>
+      <c r="F32" s="2" t="inlineStr">
+        <is>
+          <t>ad-network landing page / blog</t>
+        </is>
+      </c>
+      <c r="G32" s="2" t="inlineStr">
+        <is>
+          <t>buy traffic / choose platform</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -976,6 +1464,21 @@
       <c r="D33" s="2" t="n">
         <v>160</v>
       </c>
+      <c r="E33" s="3" t="inlineStr">
+        <is>
+          <t>Agency landing pages rank despite tiny authority (bvcompany.org DR5 holds #1 and #10, Square in the Air DR31, Samba Digital) beside the Semrush agency directory, Sportradar's services page and LinkedIn Pulse UGC — a notably weak SERP.</t>
+        </is>
+      </c>
+      <c r="F33" s="2" t="inlineStr">
+        <is>
+          <t>agency landing page</t>
+        </is>
+      </c>
+      <c r="G33" s="2" t="inlineStr">
+        <is>
+          <t>choose vendor/tool</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -992,6 +1495,21 @@
       <c r="D34" s="2" t="n">
         <v>160</v>
       </c>
+      <c r="E34" s="3" t="inlineStr">
+        <is>
+          <t>Affiliate directories win (iGB Affiliate directory, AffCatalog, AffPapa, DR21 AffSecret, aff.studio) plus a RichAds listicle; Reddit sits at #5. Directory format plus mid-DR field.</t>
+        </is>
+      </c>
+      <c r="F34" s="2" t="inlineStr">
+        <is>
+          <t>program directory</t>
+        </is>
+      </c>
+      <c r="G34" s="2" t="inlineStr">
+        <is>
+          <t>join affiliate program</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -1008,6 +1526,21 @@
       <c r="D35" s="2" t="n">
         <v>160</v>
       </c>
+      <c r="E35" s="3" t="inlineStr">
+        <is>
+          <t>Vendor product/solution pages rank (OptiKPI, Wizards, Kanggiten, Optimove) alongside a Track360 guide, but the SERP is strikingly weak: DR1 icatalyft at #2, DR4.7 cognaix, and a LinkedIn job posting all crack the top 10.</t>
+        </is>
+      </c>
+      <c r="F35" s="2" t="inlineStr">
+        <is>
+          <t>product landing page</t>
+        </is>
+      </c>
+      <c r="G35" s="2" t="inlineStr">
+        <is>
+          <t>choose vendor/tool</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -1024,6 +1557,21 @@
       <c r="D36" s="2" t="n">
         <v>140</v>
       </c>
+      <c r="E36" s="3" t="inlineStr">
+        <is>
+          <t>Casino-SEO agency landing pages win, including exact-match low-DR domains (seocasinomarketing.com DR3.1, seo.casino, DR3 Marqade) plus GeekyTech and directories (Semrush, DesignRush); a LinkedIn company page ranks #2 — soft SERP.</t>
+        </is>
+      </c>
+      <c r="F36" s="2" t="inlineStr">
+        <is>
+          <t>agency landing page</t>
+        </is>
+      </c>
+      <c r="G36" s="2" t="inlineStr">
+        <is>
+          <t>choose vendor/tool</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -1040,6 +1588,21 @@
       <c r="D37" s="2" t="n">
         <v>100</v>
       </c>
+      <c r="E37" s="3" t="inlineStr">
+        <is>
+          <t>Meta's own properties dominate — three facebook.com help/business pages plus transparency.meta ad standards — with a Hunch how-to, GambleAware and Rest of World coverage; Reddit and BlackHatWorld UGC also rank.</t>
+        </is>
+      </c>
+      <c r="F37" s="2" t="inlineStr">
+        <is>
+          <t>policy documentation</t>
+        </is>
+      </c>
+      <c r="G37" s="2" t="inlineStr">
+        <is>
+          <t>policy / compliance reference</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -1056,6 +1619,21 @@
       <c r="D38" s="2" t="n">
         <v>100</v>
       </c>
+      <c r="E38" s="3" t="inlineStr">
+        <is>
+          <t>Email SaaS vendors win with industry solution pages and strategy guides (iPost holds three slots, UniOne, Selzy, Litmus, Evenbet); low-DR guides (DR7 Casino Marketing Bootcamp, DR16 Marketing Results) and a YouTube video also rank.</t>
+        </is>
+      </c>
+      <c r="F38" s="2" t="inlineStr">
+        <is>
+          <t>vendor solution page / guide</t>
+        </is>
+      </c>
+      <c r="G38" s="2" t="inlineStr">
+        <is>
+          <t>mixed</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -1072,6 +1650,21 @@
       <c r="D39" s="2" t="n">
         <v>100</v>
       </c>
+      <c r="E39" s="3" t="inlineStr">
+        <is>
+          <t>Platform providers' product pages lead (Aristocrat Interactive #1, Gamingtec, BetConstruct, DR0.5 OHS Gaming) with provider listicles (Kodedice, AllinAffiliates, Smartico) and a SoftSwiss definition page; Reddit and LinkedIn UGC appear low in the top 10.</t>
+        </is>
+      </c>
+      <c r="F39" s="2" t="inlineStr">
+        <is>
+          <t>product landing page</t>
+        </is>
+      </c>
+      <c r="G39" s="2" t="inlineStr">
+        <is>
+          <t>choose vendor/tool</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -1088,6 +1681,21 @@
       <c r="D40" s="2" t="n">
         <v>100</v>
       </c>
+      <c r="E40" s="3" t="inlineStr">
+        <is>
+          <t>Land-based casino-management software SERP: a SoftwareReviews category page at #1, vendor product pages (Agilysys, Infor, CT Gaming, DR9 MRI AIM, DR21 Playersoft) and a Smartico listicle; YouTube ranks #9. Skews CMS/ops, not advertising.</t>
+        </is>
+      </c>
+      <c r="F40" s="2" t="inlineStr">
+        <is>
+          <t>product landing page</t>
+        </is>
+      </c>
+      <c r="G40" s="2" t="inlineStr">
+        <is>
+          <t>choose vendor/tool</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -1104,6 +1712,21 @@
       <c r="D41" s="2" t="n">
         <v>100</v>
       </c>
+      <c r="E41" s="3" t="inlineStr">
+        <is>
+          <t>Totally fragmented, non-advertising SERP: foot-traffic sensor vendor (#1 Sensource), local news traffic plans, weather cams, three YouTube results, Trustpilot, and 'betting on live traffic' novelty coverage. No advertiser intent visible.</t>
+        </is>
+      </c>
+      <c r="F41" s="2" t="inlineStr">
+        <is>
+          <t>mixed/fragmented</t>
+        </is>
+      </c>
+      <c r="G41" s="2" t="inlineStr">
+        <is>
+          <t>mixed</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -1120,6 +1743,21 @@
       <c r="D42" s="2" t="n">
         <v>100</v>
       </c>
+      <c r="E42" s="3" t="inlineStr">
+        <is>
+          <t>B2B SaaS and consultancy blog thought-leadership sweeps the SERP (Optimove, Dynamic Yield, Intellias, Symphony Solutions, Nuxgame, Track360, DR26 Rapidpace); one LinkedIn Pulse UGC result. Pure vendor-education play.</t>
+        </is>
+      </c>
+      <c r="F42" s="2" t="inlineStr">
+        <is>
+          <t>vendor blog article</t>
+        </is>
+      </c>
+      <c r="G42" s="2" t="inlineStr">
+        <is>
+          <t>learn / how-to</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -1136,6 +1774,21 @@
       <c r="D43" s="2" t="n">
         <v>90</v>
       </c>
+      <c r="E43" s="3" t="inlineStr">
+        <is>
+          <t>Affiliate networks' own pages (Gambling-Affiliation, n1.partners), directories (iGB Affiliate, DR13 AffCaptain) and listicles from ad-tech blogs (RichAds, Voluum) share the SERP with a Paysafe resource page; Reddit ranks #3.</t>
+        </is>
+      </c>
+      <c r="F43" s="2" t="inlineStr">
+        <is>
+          <t>directory / listicle</t>
+        </is>
+      </c>
+      <c r="G43" s="2" t="inlineStr">
+        <is>
+          <t>join affiliate program</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -1152,6 +1805,21 @@
       <c r="D44" s="2" t="n">
         <v>90</v>
       </c>
+      <c r="E44" s="3" t="inlineStr">
+        <is>
+          <t>Split-intent oddity: 'traffic betting' novelty content (Reddit #2, Trustpilot review of cctv-game.live, Instagram, Bitcointalk, Sigma news) collides with ad-network pages (RichAds /betting-traffic LP, TrafficGuard). Heavy UGC and no settled meaning.</t>
+        </is>
+      </c>
+      <c r="F44" s="2" t="inlineStr">
+        <is>
+          <t>mixed/fragmented</t>
+        </is>
+      </c>
+      <c r="G44" s="2" t="inlineStr">
+        <is>
+          <t>mixed</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -1168,6 +1836,21 @@
       <c r="D45" s="2" t="n">
         <v>90</v>
       </c>
+      <c r="E45" s="3" t="inlineStr">
+        <is>
+          <t>Trend-report articles from iGaming platform vendors win (Kodedice, Rapyd, SoftSwiss report, Symphony Solutions, RichAds) plus the AGA revenue tracker and a LinkedIn Pulse piece — annual-roundup reference content.</t>
+        </is>
+      </c>
+      <c r="F45" s="2" t="inlineStr">
+        <is>
+          <t>trend report / blog</t>
+        </is>
+      </c>
+      <c r="G45" s="2" t="inlineStr">
+        <is>
+          <t>industry reference</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -1184,6 +1867,21 @@
       <c r="D46" s="2" t="n">
         <v>80</v>
       </c>
+      <c r="E46" s="3" t="inlineStr">
+        <is>
+          <t>Affiliate-SaaS vendor blog and glossary pages dominate (Track360 holds three slots, DR16 Intelitics, Affilka, Post Affiliate Pro) with the StatsDrone directory and a 1xBet affiliates post — vendor-education SERP with modest competition.</t>
+        </is>
+      </c>
+      <c r="F46" s="2" t="inlineStr">
+        <is>
+          <t>vendor blog / glossary</t>
+        </is>
+      </c>
+      <c r="G46" s="2" t="inlineStr">
+        <is>
+          <t>choose vendor/tool</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -1200,6 +1898,21 @@
       <c r="D47" s="2" t="n">
         <v>70</v>
       </c>
+      <c r="E47" s="3" t="inlineStr">
+        <is>
+          <t>Ad networks win with vertical landing pages (Pushground, AADS) and how-to blogs (Voluum, RichAds, Adcash); X's gambling ads policy, Reddit, Instagram, and a spammy stck.me post also rank — commercial SERP with soft spots.</t>
+        </is>
+      </c>
+      <c r="F47" s="2" t="inlineStr">
+        <is>
+          <t>ad-network landing page / blog</t>
+        </is>
+      </c>
+      <c r="G47" s="2" t="inlineStr">
+        <is>
+          <t>buy traffic / choose platform</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -1216,6 +1929,21 @@
       <c r="D48" s="2" t="n">
         <v>70</v>
       </c>
+      <c r="E48" s="3" t="inlineStr">
+        <is>
+          <t>Mixed authority SERP: legal/research pieces lead (IMGL magazine #1, Greo, NIH) followed by agency pages (DR37 Famesters, Luvkaizen), an influencer list (Viral Nation), the Semrush directory, and LinkedIn/Reddit UGC.</t>
+        </is>
+      </c>
+      <c r="F48" s="2" t="inlineStr">
+        <is>
+          <t>mixed/fragmented</t>
+        </is>
+      </c>
+      <c r="G48" s="2" t="inlineStr">
+        <is>
+          <t>mixed</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -1232,6 +1960,21 @@
       <c r="D49" s="2" t="n">
         <v>70</v>
       </c>
+      <c r="E49" s="3" t="inlineStr">
+        <is>
+          <t>Regulators and industry bodies own it: NY Gaming Commission #1, Mass.gov regulation text, AGA marketing code, Meta ad standards, plus ESPN news and a law-school analysis. Nearly all DR70-92 — a true compliance-reference SERP.</t>
+        </is>
+      </c>
+      <c r="F49" s="2" t="inlineStr">
+        <is>
+          <t>policy documentation</t>
+        </is>
+      </c>
+      <c r="G49" s="2" t="inlineStr">
+        <is>
+          <t>policy / compliance reference</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -1248,6 +1991,21 @@
       <c r="D50" s="2" t="n">
         <v>70</v>
       </c>
+      <c r="E50" s="3" t="inlineStr">
+        <is>
+          <t>Ad-network 'where to buy iGaming traffic' blog guides dominate (PropellerAds, AdRoll, seo.casino, Z2A) plus traffic landing pages (ReachEffect, HilltopAds); Quora is the lone UGC entry. Directly monetizable buy-traffic SERP.</t>
+        </is>
+      </c>
+      <c r="F50" s="2" t="inlineStr">
+        <is>
+          <t>ad-network blog guide</t>
+        </is>
+      </c>
+      <c r="G50" s="2" t="inlineStr">
+        <is>
+          <t>buy traffic / choose platform</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -1264,6 +2022,21 @@
       <c r="D51" s="2" t="n">
         <v>70</v>
       </c>
+      <c r="E51" s="3" t="inlineStr">
+        <is>
+          <t>Meta's own policy/help pages hold multiple slots (facebook.com #1, two transparency.meta pages) with trade news filling the rest (SBC Americas, iGaming Expert, Reuters) and a LinkedIn post; policy-doc-plus-news SERP.</t>
+        </is>
+      </c>
+      <c r="F51" s="2" t="inlineStr">
+        <is>
+          <t>policy documentation + news</t>
+        </is>
+      </c>
+      <c r="G51" s="2" t="inlineStr">
+        <is>
+          <t>policy / compliance reference</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -1280,6 +2053,21 @@
       <c r="D52" s="2" t="n">
         <v>60</v>
       </c>
+      <c r="E52" s="3" t="inlineStr">
+        <is>
+          <t>Fragmented: a Behance creative gallery at #1, blockchain-ads.com's own crypto-gambling LP at #4, AADS's casino-advertising LP, near-zero-DR marketing blogs (Adspires DR0, Scale with Ascend DR0, Coinpresso DR26), Rolling Stone news and Reddit. Weak, unconsolidated SERP BCA already touches.</t>
+        </is>
+      </c>
+      <c r="F52" s="2" t="inlineStr">
+        <is>
+          <t>mixed/fragmented</t>
+        </is>
+      </c>
+      <c r="G52" s="2" t="inlineStr">
+        <is>
+          <t>mixed</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -1296,6 +2084,21 @@
       <c r="D53" s="2" t="n">
         <v>60</v>
       </c>
+      <c r="E53" s="3" t="inlineStr">
+        <is>
+          <t>Industry-body guidelines and policy docs win: IAB creative-guidelines PDF, Ad Standards Canada, AGA marketing code, Meta ad standards, plus BusinessofApps' creative best-practices post and an NIH paper; one DR22 agency post ranks.</t>
+        </is>
+      </c>
+      <c r="F53" s="2" t="inlineStr">
+        <is>
+          <t>guidelines documentation</t>
+        </is>
+      </c>
+      <c r="G53" s="2" t="inlineStr">
+        <is>
+          <t>policy / compliance reference</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -1312,6 +2115,21 @@
       <c r="D54" s="2" t="n">
         <v>60</v>
       </c>
+      <c r="E54" s="3" t="inlineStr">
+        <is>
+          <t>SaaS vendors dominate: tracker/CRM product pages (voluum.com, optimove.com, bloomreach.com) mixed with affiliate-software vendor blogs (track360.io, affise.com, irev.com, aff.tech) and an f6s.com software directory. All commercial DR 30-83, no UGC.</t>
+        </is>
+      </c>
+      <c r="F54" s="2" t="inlineStr">
+        <is>
+          <t>product landing page</t>
+        </is>
+      </c>
+      <c r="G54" s="2" t="inlineStr">
+        <is>
+          <t>choose vendor/tool</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -1328,6 +2146,21 @@
       <c r="D55" s="2" t="n">
         <v>60</v>
       </c>
+      <c r="E55" s="3" t="inlineStr">
+        <is>
+          <t>Mix of affiliate-program listicles (track360.io, businessofapps.com, affpapa.com), program signup/landing pages of operators (n1.partners, starzpartners.com, cloudbet.com/affiliates) and the affpaying.com directory; a Reddit thread ranks #2, signalling a beatable SERP with mid-DR players (DR 37-86).</t>
+        </is>
+      </c>
+      <c r="F55" s="2" t="inlineStr">
+        <is>
+          <t>listicle + program signup pages</t>
+        </is>
+      </c>
+      <c r="G55" s="2" t="inlineStr">
+        <is>
+          <t>join affiliate program</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -1344,6 +2177,21 @@
       <c r="D56" s="2" t="n">
         <v>50</v>
       </c>
+      <c r="E56" s="3" t="inlineStr">
+        <is>
+          <t>Push/pop ad-network blogs own this SERP: richads.com case studies and guides, pushground.com and roiads.co landing/blog pages, adcash.com; heavy UGC presence (Reddit r/PPC, afflift forum, YouTube) shows low competition. Format is how-to/case-study blog posts from networks selling the traffic.</t>
+        </is>
+      </c>
+      <c r="F56" s="2" t="inlineStr">
+        <is>
+          <t>ad-network blog guide</t>
+        </is>
+      </c>
+      <c r="G56" s="2" t="inlineStr">
+        <is>
+          <t>buy traffic / choose platform</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
@@ -1360,6 +2208,21 @@
       <c r="D57" s="2" t="n">
         <v>50</v>
       </c>
+      <c r="E57" s="3" t="inlineStr">
+        <is>
+          <t>Ad-network 'best gambling ad networks' listicles dominate (richads.com, blockchain-ads.com already at #3, hilltopads.com, trafficnomads.com, betconstruct.com) alongside network landing pages (aads.com, pushground.com, reacheffect.com); Reddit and LinkedIn UGC in top 10 confirm a soft SERP.</t>
+        </is>
+      </c>
+      <c r="F57" s="2" t="inlineStr">
+        <is>
+          <t>blog listicle</t>
+        </is>
+      </c>
+      <c r="G57" s="2" t="inlineStr">
+        <is>
+          <t>buy traffic / choose platform</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -1376,6 +2239,21 @@
       <c r="D58" s="2" t="n">
         <v>50</v>
       </c>
+      <c r="E58" s="3" t="inlineStr">
+        <is>
+          <t>Fragmented SERP of crypto-marketing agency landing pages (coinpresso.io, seo.casino), ad-network product pages (aads.com, cointraffic.com), affiliate blog guides (affpapa.com, scaleo.io) and a gpwa.org forum thread at #3; many low-DR sites (DR 16-38) and forum/YouTube UGC signal weak competition.</t>
+        </is>
+      </c>
+      <c r="F58" s="2" t="inlineStr">
+        <is>
+          <t>mixed/fragmented</t>
+        </is>
+      </c>
+      <c r="G58" s="2" t="inlineStr">
+        <is>
+          <t>buy traffic / choose platform</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="inlineStr">
@@ -1392,6 +2270,21 @@
       <c r="D59" s="2" t="n">
         <v>40</v>
       </c>
+      <c r="E59" s="3" t="inlineStr">
+        <is>
+          <t>Affiliate-software and tracker blogs (track360.io, irev.com, voluum.com, affnook.com, maxweb.com, partnermatrix.com) publish benchmark/data posts; very low-DR pages rank high (redclawey.com DR 10 at #2, smsedge.com DR 8) plus YouTube/Reddit UGC — a soft data-driven SERP.</t>
+        </is>
+      </c>
+      <c r="F59" s="2" t="inlineStr">
+        <is>
+          <t>data/benchmark blog post</t>
+        </is>
+      </c>
+      <c r="G59" s="2" t="inlineStr">
+        <is>
+          <t>learn / how-to</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -1408,6 +2301,21 @@
       <c r="D60" s="2" t="n">
         <v>40</v>
       </c>
+      <c r="E60" s="3" t="inlineStr">
+        <is>
+          <t>PPC agency service pages (elit-web.com, optimum7.com, ppcjuice.com, circusppc.com, wiredmedia.co.uk) and agency-directory listings (clutch.co DR 91) compete with tracker blogs (voluum.com, clickguard.com, propellerads.com); LinkedIn UGC and DR 3-15 domains in top 10 show weakness.</t>
+        </is>
+      </c>
+      <c r="F60" s="2" t="inlineStr">
+        <is>
+          <t>agency service page</t>
+        </is>
+      </c>
+      <c r="G60" s="2" t="inlineStr">
+        <is>
+          <t>choose vendor/tool</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
@@ -1424,6 +2332,21 @@
       <c r="D61" s="2" t="n">
         <v>40</v>
       </c>
+      <c r="E61" s="3" t="inlineStr">
+        <is>
+          <t>Google's own policy documentation ranks #1 (support.google.com DR 99) but the rest is thin: a Reddit AMA at #2, low-DR agency pages (ppcjuice.com DR 3), tracker blog (voluum.com) and LinkedIn posts — very shallow SERP beyond the policy page.</t>
+        </is>
+      </c>
+      <c r="F61" s="2" t="inlineStr">
+        <is>
+          <t>policy doc + how-to guides</t>
+        </is>
+      </c>
+      <c r="G61" s="2" t="inlineStr">
+        <is>
+          <t>learn / how-to</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -1440,6 +2363,21 @@
       <c r="D62" s="2" t="n">
         <v>40</v>
       </c>
+      <c r="E62" s="3" t="inlineStr">
+        <is>
+          <t>TikTok's own help-center policy articles occupy most positions (ads.tiktok.com help pages), padded by BlackHatWorld and Reddit threads and one DR 32 blog guide — platform documentation is the answer, with only UGC as third-party competition.</t>
+        </is>
+      </c>
+      <c r="F62" s="2" t="inlineStr">
+        <is>
+          <t>policy documentation</t>
+        </is>
+      </c>
+      <c r="G62" s="2" t="inlineStr">
+        <is>
+          <t>policy / compliance reference</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
@@ -1456,6 +2394,21 @@
       <c r="D63" s="2" t="n">
         <v>40</v>
       </c>
+      <c r="E63" s="3" t="inlineStr">
+        <is>
+          <t>All high-DR authority: regulators and industry bodies (gamblingcommission.gov.uk, americangaming.org, bettingandgamingcouncil.com, massgaming.com), academic papers (pmc.ncbi.nlm.nih.gov) and research PDFs. Zero commercial players and zero UGC — a hard, informational/regulatory SERP.</t>
+        </is>
+      </c>
+      <c r="F63" s="2" t="inlineStr">
+        <is>
+          <t>policy documentation</t>
+        </is>
+      </c>
+      <c r="G63" s="2" t="inlineStr">
+        <is>
+          <t>policy / compliance reference</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -1472,6 +2425,21 @@
       <c r="D64" s="2" t="n">
         <v>40</v>
       </c>
+      <c r="E64" s="3" t="inlineStr">
+        <is>
+          <t>Affiliate directories and listicles (businessofapps.com, zorbasmedia.com, 1xbetaffiliates.net) mixed with explainer posts on CPA-vs-revshare from affiliate-software vendors (track360.io, irev.com) and operator program blogs (n1.partners, roiads.co); one Reddit thread in top 10.</t>
+        </is>
+      </c>
+      <c r="F64" s="2" t="inlineStr">
+        <is>
+          <t>listicle + explainer post</t>
+        </is>
+      </c>
+      <c r="G64" s="2" t="inlineStr">
+        <is>
+          <t>join affiliate program</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
@@ -1488,6 +2456,21 @@
       <c r="D65" s="2" t="n">
         <v>40</v>
       </c>
+      <c r="E65" s="3" t="inlineStr">
+        <is>
+          <t>A Reddit thread ranks #1, followed by affiliate-program directories (affpaying.com, postaffiliatepro.com, 15m.com), listicles (affpapa.com, affnook.com) and direct program signup pages (alpha-affiliates.com, nowpayments.io) — directory/listing formats win on a soft SERP.</t>
+        </is>
+      </c>
+      <c r="F65" s="2" t="inlineStr">
+        <is>
+          <t>program directory/listicle</t>
+        </is>
+      </c>
+      <c r="G65" s="2" t="inlineStr">
+        <is>
+          <t>join affiliate program</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -1504,6 +2487,21 @@
       <c r="D66" s="2" t="n">
         <v>40</v>
       </c>
+      <c r="E66" s="3" t="inlineStr">
+        <is>
+          <t>Fragmented mix of small casino-marketing agencies (vallomedia.com DR 27, playerperformancegroup.com DR 19) and general casino-marketing strategy guides (moengage.com, alphametic.com, elit-web.com), plus a LinkedIn post and casinovendors.com directory listing — no dominant format, mostly land-based casino angle.</t>
+        </is>
+      </c>
+      <c r="F66" s="2" t="inlineStr">
+        <is>
+          <t>mixed/fragmented</t>
+        </is>
+      </c>
+      <c r="G66" s="2" t="inlineStr">
+        <is>
+          <t>learn / how-to</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
@@ -1520,6 +2518,21 @@
       <c r="D67" s="2" t="n">
         <v>40</v>
       </c>
+      <c r="E67" s="3" t="inlineStr">
+        <is>
+          <t>B2B iGaming supplier pages and blogs (sportradar.com, netrefer.com, theaffiliateplatform.com, igaming.createit.com) mixed with off-topic results (law firm M&amp;A page, Wikipedia, Quora, investor news) — an unfocused SERP where strategy-guide content from platform vendors wins.</t>
+        </is>
+      </c>
+      <c r="F67" s="2" t="inlineStr">
+        <is>
+          <t>vendor blog guide</t>
+        </is>
+      </c>
+      <c r="G67" s="2" t="inlineStr">
+        <is>
+          <t>learn / how-to</t>
+        </is>
+      </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
@@ -1536,6 +2549,21 @@
       <c r="D68" s="2" t="n">
         <v>30</v>
       </c>
+      <c r="E68" s="3" t="inlineStr">
+        <is>
+          <t>Very weak SERP: DR 0-26 sites (affiliace.digital, rapidpace.com, marqade.com) plus LinkedIn/Quora/YouTube UGC rank alongside ad-network blog guides (richads.com, reacheffect.com, voluum.com); conversion/how-to blog posts win with almost no authority competition.</t>
+        </is>
+      </c>
+      <c r="F68" s="2" t="inlineStr">
+        <is>
+          <t>how-to guide</t>
+        </is>
+      </c>
+      <c r="G68" s="2" t="inlineStr">
+        <is>
+          <t>learn / how-to</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
@@ -1552,6 +2580,21 @@
       <c r="D69" s="2" t="n">
         <v>30</v>
       </c>
+      <c r="E69" s="3" t="inlineStr">
+        <is>
+          <t>Affiliate-network and tracker blogs (tracknow.io, roiads.co, richads.com, betting.partners, pmaffiliates.com) publish traffic-source guides; affiliatefix forum thread and Reddit in top 10 plus a DR 6 site show low competition.</t>
+        </is>
+      </c>
+      <c r="F69" s="2" t="inlineStr">
+        <is>
+          <t>blog guide (traffic sources)</t>
+        </is>
+      </c>
+      <c r="G69" s="2" t="inlineStr">
+        <is>
+          <t>learn / how-to</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
@@ -1568,6 +2611,21 @@
       <c r="D70" s="2" t="n">
         <v>30</v>
       </c>
+      <c r="E70" s="3" t="inlineStr">
+        <is>
+          <t>Fragmented: job listings (indeed.com), Reddit thread, casinovendors.com supplier directory, agency pages (bird.marketing, designrush.com directory) and iGaming media-buying guides (affise.com, betboyz.com DR 13); no clear winning format — intent splits between hiring, agencies and how-to.</t>
+        </is>
+      </c>
+      <c r="F70" s="2" t="inlineStr">
+        <is>
+          <t>mixed/fragmented</t>
+        </is>
+      </c>
+      <c r="G70" s="2" t="inlineStr">
+        <is>
+          <t>mixed</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
@@ -1584,6 +2642,21 @@
       <c r="D71" s="2" t="n">
         <v>30</v>
       </c>
+      <c r="E71" s="3" t="inlineStr">
+        <is>
+          <t>Split between high-DR policy/regulatory pages (support.google.com, transparency.meta.com, gamblingcommission.gov.uk, an NCBI paper) and practitioner guides from agencies/media (tegna.com, elit-web.com, licensegentlemen.com); a Reddit AMA sits in the top 10. Compliance-aware best-practice guides win.</t>
+        </is>
+      </c>
+      <c r="F71" s="2" t="inlineStr">
+        <is>
+          <t>how-to guide + policy docs</t>
+        </is>
+      </c>
+      <c r="G71" s="2" t="inlineStr">
+        <is>
+          <t>learn / how-to</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -1600,6 +2673,21 @@
       <c r="D72" s="2" t="n">
         <v>30</v>
       </c>
+      <c r="E72" s="3" t="inlineStr">
+        <is>
+          <t>Affiliate-tooling vendors and directories rank: businessofapps.com casino list at #1, tracking-software pages (trafficmanager.com, affilka.com), tool listicles (smartico.ai, allinaffiliates.com DR 12) and ad-network blogs (richads.com); Quora and Reddit UGC in top 10 signal softness.</t>
+        </is>
+      </c>
+      <c r="F72" s="2" t="inlineStr">
+        <is>
+          <t>tool listicle</t>
+        </is>
+      </c>
+      <c r="G72" s="2" t="inlineStr">
+        <is>
+          <t>choose vendor/tool</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
@@ -1616,6 +2704,21 @@
       <c r="D73" s="2" t="n">
         <v>30</v>
       </c>
+      <c r="E73" s="3" t="inlineStr">
+        <is>
+          <t>Competitor ad-network listicles (richads.com, monetag.com, propellerads.com) and software-review directories (capterra.com DR 91) compete with Adsterra's own 'alternatives' blog posts ranking for its brand; one Reddit thread. Classic alternatives-listicle SERP.</t>
+        </is>
+      </c>
+      <c r="F73" s="2" t="inlineStr">
+        <is>
+          <t>alternatives listicle</t>
+        </is>
+      </c>
+      <c r="G73" s="2" t="inlineStr">
+        <is>
+          <t>compare options (listicle)</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
@@ -1632,6 +2735,21 @@
       <c r="D74" s="2" t="n">
         <v>30</v>
       </c>
+      <c r="E74" s="3" t="inlineStr">
+        <is>
+          <t>Very weak SERP: influencer-agency landing pages and blogs (famesters.com DR 37, luvkaizen.com, awisee.com) mixed with DR 0.7-16 blogs, Reddit and LinkedIn UGC — no authority owns this; agency service pages and guides both rank.</t>
+        </is>
+      </c>
+      <c r="F74" s="2" t="inlineStr">
+        <is>
+          <t>agency page / blog guide</t>
+        </is>
+      </c>
+      <c r="G74" s="2" t="inlineStr">
+        <is>
+          <t>learn / how-to</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
@@ -1648,6 +2766,21 @@
       <c r="D75" s="2" t="n">
         <v>30</v>
       </c>
+      <c r="E75" s="3" t="inlineStr">
+        <is>
+          <t>Long-form 'complete guide' blog posts from affiliate-software and ad-network vendors (tracknow.io, irev.com, richads.com, bloomreach.com gated guide) plus low-DR agency blogs (rainmakeragency.ai, smsedge.com DR 8, envisioner.io DR 14) — beatable guide-format SERP.</t>
+        </is>
+      </c>
+      <c r="F75" s="2" t="inlineStr">
+        <is>
+          <t>long-form guide</t>
+        </is>
+      </c>
+      <c r="G75" s="2" t="inlineStr">
+        <is>
+          <t>learn / how-to</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
@@ -1664,6 +2797,21 @@
       <c r="D76" s="2" t="n">
         <v>30</v>
       </c>
+      <c r="E76" s="3" t="inlineStr">
+        <is>
+          <t>Dominated by academic and public-interest research (bristol.ac.uk report, Springer, NCBI, theguardian.com, bi.team, greo.ca) on gambling-ad harms plus Meta's help page — a high-DR harm-focused informational SERP, not a practitioner one; hard for commercial content.</t>
+        </is>
+      </c>
+      <c r="F76" s="2" t="inlineStr">
+        <is>
+          <t>research report/news</t>
+        </is>
+      </c>
+      <c r="G76" s="2" t="inlineStr">
+        <is>
+          <t>industry reference</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
@@ -1680,6 +2828,21 @@
       <c r="D77" s="2" t="n">
         <v>30</v>
       </c>
+      <c r="E77" s="3" t="inlineStr">
+        <is>
+          <t>A DR 2.6 agency page ranks #1 (tentenseven.com) ahead of industry-body data (americangaming.org), vendor strategy blogs (tecpinion.com, gammastack.com, optimove.com, richads.com) and a LinkedIn post at #2 — extremely soft SERP won by strategy guides and agency pages.</t>
+        </is>
+      </c>
+      <c r="F77" s="2" t="inlineStr">
+        <is>
+          <t>strategy blog guide</t>
+        </is>
+      </c>
+      <c r="G77" s="2" t="inlineStr">
+        <is>
+          <t>learn / how-to</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
@@ -1696,6 +2859,21 @@
       <c r="D78" s="2" t="n">
         <v>20</v>
       </c>
+      <c r="E78" s="3" t="inlineStr">
+        <is>
+          <t>Casino-marketing strategy guides from agencies and martech vendors (alphametic.com, elit-web.com, selzy.com, moengage.com, cvent.com, scaleo.io funnel post); #1 is a DR 24 blog (translationroyale.com) and YouTube ranks mid-page — funnel/strategy blog posts win a soft SERP.</t>
+        </is>
+      </c>
+      <c r="F78" s="2" t="inlineStr">
+        <is>
+          <t>strategy blog guide</t>
+        </is>
+      </c>
+      <c r="G78" s="2" t="inlineStr">
+        <is>
+          <t>learn / how-to</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
@@ -1712,6 +2890,21 @@
       <c r="D79" s="2" t="n">
         <v>20</v>
       </c>
+      <c r="E79" s="3" t="inlineStr">
+        <is>
+          <t>Explainer posts from affiliate-software vendors (track360.io, irev.com, voluum.com, affcatalog.com glossary) plus businessofapps.com revshare listicle and richads.com program listicle; LinkedIn and Reddit UGC in top 10.</t>
+        </is>
+      </c>
+      <c r="F79" s="2" t="inlineStr">
+        <is>
+          <t>explainer blog post</t>
+        </is>
+      </c>
+      <c r="G79" s="2" t="inlineStr">
+        <is>
+          <t>learn / how-to</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
@@ -1728,6 +2921,21 @@
       <c r="D80" s="2" t="n">
         <v>20</v>
       </c>
+      <c r="E80" s="3" t="inlineStr">
+        <is>
+          <t>Small specialist agency pages (andava.com, socialtrend.co.uk, luvkaizen.com) and vendor blog tips (incomeaccess.com, bgaming.com, voluum.com) with a LinkedIn article at #3 — low-competition SERP split between agency service pages and tips posts.</t>
+        </is>
+      </c>
+      <c r="F80" s="2" t="inlineStr">
+        <is>
+          <t>agency page / tips post</t>
+        </is>
+      </c>
+      <c r="G80" s="2" t="inlineStr">
+        <is>
+          <t>learn / how-to</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
@@ -1744,6 +2952,21 @@
       <c r="D81" s="2" t="n">
         <v>20</v>
       </c>
+      <c r="E81" s="3" t="inlineStr">
+        <is>
+          <t>Fragmented: agency directories (agencies.semrush.com, topdevelopers.co), academic papers (NCBI, sciencedirect.com), strategy blogs (aads.com, alphametic.com) and SaaS solution pages (optimove.com) — mixed intent with no dominant format.</t>
+        </is>
+      </c>
+      <c r="F81" s="2" t="inlineStr">
+        <is>
+          <t>mixed/fragmented</t>
+        </is>
+      </c>
+      <c r="G81" s="2" t="inlineStr">
+        <is>
+          <t>mixed</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
@@ -1760,6 +2983,21 @@
       <c r="D82" s="2" t="n">
         <v>20</v>
       </c>
+      <c r="E82" s="3" t="inlineStr">
+        <is>
+          <t>Program directories and listicles win: businessofapps.com, mylead.global, zorbasmedia.com, 15m.com, plus track360.io educational hub pages and goaffiliates.com signup page at #1 (DR 39); a Reddit thread at #2 shows softness.</t>
+        </is>
+      </c>
+      <c r="F82" s="2" t="inlineStr">
+        <is>
+          <t>program directory/listicle</t>
+        </is>
+      </c>
+      <c r="G82" s="2" t="inlineStr">
+        <is>
+          <t>join affiliate program</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
@@ -1776,6 +3014,21 @@
       <c r="D83" s="2" t="n">
         <v>20</v>
       </c>
+      <c r="E83" s="3" t="inlineStr">
+        <is>
+          <t>Retention/acquisition strategy blog posts from iGaming platform vendors and agencies (selzy.com, everymatrix.com, lt.agency, moengage.com, track360.io glossary); YouTube and Quora UGC in the top 10 and low-DR entrants (envisioner.io DR 14) make it beatable.</t>
+        </is>
+      </c>
+      <c r="F83" s="2" t="inlineStr">
+        <is>
+          <t>strategy blog guide</t>
+        </is>
+      </c>
+      <c r="G83" s="2" t="inlineStr">
+        <is>
+          <t>learn / how-to</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
@@ -1792,6 +3045,21 @@
       <c r="D84" s="2" t="n">
         <v>20</v>
       </c>
+      <c r="E84" s="3" t="inlineStr">
+        <is>
+          <t>Research and news dominate (bristol.ac.uk, NCBI, norc.org, espn.com) but practitioner content ranks too (contentstadium.com content-ideas post, smartico.ai strategies, elit-web.com) — hybrid SERP leaning informational with high-DR studies.</t>
+        </is>
+      </c>
+      <c r="F84" s="2" t="inlineStr">
+        <is>
+          <t>research + strategy posts</t>
+        </is>
+      </c>
+      <c r="G84" s="2" t="inlineStr">
+        <is>
+          <t>learn / how-to</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
@@ -1808,6 +3076,21 @@
       <c r="D85" s="2" t="n">
         <v>20</v>
       </c>
+      <c r="E85" s="3" t="inlineStr">
+        <is>
+          <t>B2B esports-odds and platform vendors (oddin.gg, gr8.tech, rebelbetting.com), market-research reports (businessresearchinsights.com) and industry media (sigma.world, digiday.com) — all mid-to-high DR blog/strategy content, no UGC; guide posts from suppliers win.</t>
+        </is>
+      </c>
+      <c r="F85" s="2" t="inlineStr">
+        <is>
+          <t>vendor blog guide</t>
+        </is>
+      </c>
+      <c r="G85" s="2" t="inlineStr">
+        <is>
+          <t>learn / how-to</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
@@ -1824,6 +3107,21 @@
       <c r="D86" s="2" t="n">
         <v>10</v>
       </c>
+      <c r="E86" s="3" t="inlineStr">
+        <is>
+          <t>Weak, fragmented SERP: two Reddit threads and a LinkedIn company page in the top 5, job boards (indeed.com, djinni.co), one affise.com guide and a DR 13 blog at #2 — how-to content from vendors barely competes with UGC and jobs listings.</t>
+        </is>
+      </c>
+      <c r="F86" s="2" t="inlineStr">
+        <is>
+          <t>mixed/fragmented</t>
+        </is>
+      </c>
+      <c r="G86" s="2" t="inlineStr">
+        <is>
+          <t>mixed</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
@@ -1840,6 +3138,21 @@
       <c r="D87" s="2" t="n">
         <v>10</v>
       </c>
+      <c r="E87" s="3" t="inlineStr">
+        <is>
+          <t>Trend-report roundups from iGaming suppliers and ad networks (bgaming.com, richads.com, softwaremind.com, evenbetgaming.com), industry-body data (americangaming.org), appsflyer.com report and a SOFTSWISS report on Scribd — annual trends listicle format wins.</t>
+        </is>
+      </c>
+      <c r="F87" s="2" t="inlineStr">
+        <is>
+          <t>trends report/listicle</t>
+        </is>
+      </c>
+      <c r="G87" s="2" t="inlineStr">
+        <is>
+          <t>industry reference</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -1856,6 +3169,21 @@
       <c r="D88" s="2" t="n">
         <v>10</v>
       </c>
+      <c r="E88" s="3" t="inlineStr">
+        <is>
+          <t>Pop/push ad networks own the SERP with explainer and buy pages (richads.com what-is post, reacheffect.com buy-popunder page, roiads.co, activerevenue.com, kadam.net, lospollos.com) plus businessofapps.com; a BlackHatWorld thread and DR 11 site in top 10 confirm low difficulty.</t>
+        </is>
+      </c>
+      <c r="F88" s="2" t="inlineStr">
+        <is>
+          <t>ad-network explainer/landing</t>
+        </is>
+      </c>
+      <c r="G88" s="2" t="inlineStr">
+        <is>
+          <t>buy traffic / choose platform</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
@@ -1872,6 +3200,21 @@
       <c r="D89" s="2" t="n">
         <v>10</v>
       </c>
+      <c r="E89" s="3" t="inlineStr">
+        <is>
+          <t>High-DR data sources dominate: americangaming.org report and PDF at #2-3, trade press (sbcamericas.com, emarketer.com, espn.com) and statistics hubs (rg.org); LinkedIn and Facebook posts fill the tail. A stats/data-report SERP.</t>
+        </is>
+      </c>
+      <c r="F89" s="2" t="inlineStr">
+        <is>
+          <t>data report/statistics page</t>
+        </is>
+      </c>
+      <c r="G89" s="2" t="inlineStr">
+        <is>
+          <t>industry reference</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
@@ -1888,6 +3231,21 @@
       <c r="D90" s="2" t="n">
         <v>10</v>
       </c>
+      <c r="E90" s="3" t="inlineStr">
+        <is>
+          <t>Software-review directories dominate (g2.com, capterra.com, getapp.ca DR 57-91) alongside HilltopAds' own pages ranking for its brand, a comparison page (adspyglass.com) and monetag.com listicle; Reddit and YouTube in top 10.</t>
+        </is>
+      </c>
+      <c r="F90" s="2" t="inlineStr">
+        <is>
+          <t>review-directory alternatives page</t>
+        </is>
+      </c>
+      <c r="G90" s="2" t="inlineStr">
+        <is>
+          <t>compare options (listicle)</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="inlineStr">
@@ -1904,6 +3262,21 @@
       <c r="D91" s="2" t="n">
         <v>10</v>
       </c>
+      <c r="E91" s="3" t="inlineStr">
+        <is>
+          <t>PropellerAds' own domain holds four spots (its 'alternatives to X' blog posts plus homepage), with richads.com competitor listicle at #2, review directories (g2.com, cuspera.com) and a Reddit thread — alternatives listicles and review pages win.</t>
+        </is>
+      </c>
+      <c r="F91" s="2" t="inlineStr">
+        <is>
+          <t>alternatives listicle</t>
+        </is>
+      </c>
+      <c r="G91" s="2" t="inlineStr">
+        <is>
+          <t>compare options (listicle)</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
@@ -1920,6 +3293,21 @@
       <c r="D92" s="2" t="n">
         <v>10</v>
       </c>
+      <c r="E92" s="3" t="inlineStr">
+        <is>
+          <t>Regulator and industry-body documentation leads (gamblingcommission.gov.uk, americangaming.org, adstandards.ca, Xiaomi platform policy) but commercial compliance guides also rank (richads.com, adspyder.io, oddsindex.com DR 36); one Quora thread — compliance-guide content can compete.</t>
+        </is>
+      </c>
+      <c r="F92" s="2" t="inlineStr">
+        <is>
+          <t>policy docs + compliance guide</t>
+        </is>
+      </c>
+      <c r="G92" s="2" t="inlineStr">
+        <is>
+          <t>policy / compliance reference</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -1936,6 +3324,21 @@
       <c r="D93" s="2" t="n">
         <v>10</v>
       </c>
+      <c r="E93" s="3" t="inlineStr">
+        <is>
+          <t>Microsoft's own properties monopolize the SERP (about.ads.microsoft.com policy pages, forms and change logs, learn.microsoft.com — DR 96) with only searchenginejournal.com and a small consultancy commenting; effectively unwinnable brand-policy SERP.</t>
+        </is>
+      </c>
+      <c r="F93" s="2" t="inlineStr">
+        <is>
+          <t>policy documentation</t>
+        </is>
+      </c>
+      <c r="G93" s="2" t="inlineStr">
+        <is>
+          <t>policy / compliance reference</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="inlineStr">
@@ -1952,6 +3355,21 @@
       <c r="D94" s="2" t="n">
         <v>10</v>
       </c>
+      <c r="E94" s="3" t="inlineStr">
+        <is>
+          <t>Platform policy pages dominate: Taboola's own casino/gambling policy FAQ and playbook PDF, plus Meta, AdRoll and NY gaming-commission policy pages; Reddit and YouTube fill gaps — official documentation is what ranks.</t>
+        </is>
+      </c>
+      <c r="F94" s="2" t="inlineStr">
+        <is>
+          <t>policy documentation</t>
+        </is>
+      </c>
+      <c r="G94" s="2" t="inlineStr">
+        <is>
+          <t>policy / compliance reference</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
@@ -1968,6 +3386,21 @@
       <c r="D95" s="2" t="n">
         <v>10</v>
       </c>
+      <c r="E95" s="3" t="inlineStr">
+        <is>
+          <t>Fraud-prevention and KYC vendors own it with explainer blogs (group-ib.com, sumsub.com, gbg.com, paysafe.com, bluepear.net) plus affiliate-software posts (irev.com); all solid DR 38-81 except one Instagram post — educational vendor content wins.</t>
+        </is>
+      </c>
+      <c r="F95" s="2" t="inlineStr">
+        <is>
+          <t>vendor explainer post</t>
+        </is>
+      </c>
+      <c r="G95" s="2" t="inlineStr">
+        <is>
+          <t>learn / how-to</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
@@ -1984,6 +3417,21 @@
       <c r="D96" s="2" t="n">
         <v>10</v>
       </c>
+      <c r="E96" s="3" t="inlineStr">
+        <is>
+          <t>Split SERP: affiliate-marketing explainers from trackers (voluum.com #1, irev.com, richads.com) and agency pages (sambadigital.com, lengreo.com list) against job boards (ziprecruiter.com, igamingcareers.co) — guide content wins the marketing intent.</t>
+        </is>
+      </c>
+      <c r="F96" s="2" t="inlineStr">
+        <is>
+          <t>blog guide</t>
+        </is>
+      </c>
+      <c r="G96" s="2" t="inlineStr">
+        <is>
+          <t>learn / how-to</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -2000,6 +3448,21 @@
       <c r="D97" s="2" t="n">
         <v>10</v>
       </c>
+      <c r="E97" s="3" t="inlineStr">
+        <is>
+          <t>Benchmark/rate explainer posts from affiliate-software and network blogs (bigbetty.io CPA-tiers post, track360.io, partnermatrix.com, propellerads.com, voluum.com, affnook.com glossary); DR 8-13 sites rank (smsedge.com #2, affcaptain.com) — soft data-oriented SERP.</t>
+        </is>
+      </c>
+      <c r="F97" s="2" t="inlineStr">
+        <is>
+          <t>data/benchmark blog post</t>
+        </is>
+      </c>
+      <c r="G97" s="2" t="inlineStr">
+        <is>
+          <t>learn / how-to</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="inlineStr">
@@ -2016,6 +3479,21 @@
       <c r="D98" s="2" t="n">
         <v>10</v>
       </c>
+      <c r="E98" s="3" t="inlineStr">
+        <is>
+          <t>Attribution SaaS vendors rank with product/solution pages (intelitics.com DR 16, singular.net, adjust.com, violetgrowth.com) and software listicles/guides (affise.com, hockeystack.com, track360.io learn hub); low-DR specialists at the top signal a winnable vendor SERP.</t>
+        </is>
+      </c>
+      <c r="F98" s="2" t="inlineStr">
+        <is>
+          <t>product landing page</t>
+        </is>
+      </c>
+      <c r="G98" s="2" t="inlineStr">
+        <is>
+          <t>choose vendor/tool</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
@@ -2032,6 +3510,21 @@
       <c r="D99" s="2" t="n">
         <v>10</v>
       </c>
+      <c r="E99" s="3" t="inlineStr">
+        <is>
+          <t>Program directories and comparison pages (businessofapps.com, statsdrone.com, affpaying.com) plus payout-model explainers (irev.com, track360.io glossary) and a program landing page (alpha-affiliates.com); no UGC, mid-high DR.</t>
+        </is>
+      </c>
+      <c r="F99" s="2" t="inlineStr">
+        <is>
+          <t>program directory/explainer</t>
+        </is>
+      </c>
+      <c r="G99" s="2" t="inlineStr">
+        <is>
+          <t>join affiliate program</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
@@ -2048,6 +3541,21 @@
       <c r="D100" s="2" t="n">
         <v>10</v>
       </c>
+      <c r="E100" s="3" t="inlineStr">
+        <is>
+          <t>Weak SERP of crypto/iGaming agency blogs (surgence.io, coinpresso.io, kolhq.com DR 4) with blockchain-ads.com already at #6, a LinkedIn pulse at #4 and a podcast page at #3 — low-DR strategy guides win easily.</t>
+        </is>
+      </c>
+      <c r="F100" s="2" t="inlineStr">
+        <is>
+          <t>strategy blog guide</t>
+        </is>
+      </c>
+      <c r="G100" s="2" t="inlineStr">
+        <is>
+          <t>learn / how-to</t>
+        </is>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
@@ -2064,6 +3572,21 @@
       <c r="D101" s="2" t="n">
         <v>10</v>
       </c>
+      <c r="E101" s="3" t="inlineStr">
+        <is>
+          <t>Beginner-guide blog posts from affiliate software and ad networks (irev.com, richads.com, softswiss.com, statsdrone.com) plus niche sites (mercurytheme.com, highstakesdb.com, paylinedata.com); YouTube at #5 — long-form guides win.</t>
+        </is>
+      </c>
+      <c r="F101" s="2" t="inlineStr">
+        <is>
+          <t>long-form guide</t>
+        </is>
+      </c>
+      <c r="G101" s="2" t="inlineStr">
+        <is>
+          <t>learn / how-to</t>
+        </is>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
@@ -2080,6 +3603,21 @@
       <c r="D102" s="2" t="n">
         <v>10</v>
       </c>
+      <c r="E102" s="3" t="inlineStr">
+        <is>
+          <t>SMS-platform vendor pages and blogs dominate (clickatell.com, springbig.com, smsedge.com academy, texcellsms.com, optikpi.com) with a DR 11 page at #1 (mamonty.com) and LinkedIn in the tail — very soft vendor-content SERP.</t>
+        </is>
+      </c>
+      <c r="F102" s="2" t="inlineStr">
+        <is>
+          <t>vendor blog/service page</t>
+        </is>
+      </c>
+      <c r="G102" s="2" t="inlineStr">
+        <is>
+          <t>learn / how-to</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
@@ -2096,9 +3634,24 @@
       <c r="D103" s="2" t="n">
         <v>10</v>
       </c>
+      <c r="E103" s="3" t="inlineStr">
+        <is>
+          <t>Email-platform and list vendors rank (litmus.com industry page at #2, hotsol.net, mailcheck.co, dmdatabases.com list page, bvcompany.org DR 5 service page) plus a UNLV thesis and YouTube — fragmented, low-DR, easily winnable.</t>
+        </is>
+      </c>
+      <c r="F103" s="2" t="inlineStr">
+        <is>
+          <t>vendor guide/service page</t>
+        </is>
+      </c>
+      <c r="G103" s="2" t="inlineStr">
+        <is>
+          <t>learn / how-to</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D103"/>
+  <autoFilter ref="A1:G103"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>